<commit_message>
Add Email application engine, Gmail integration, batch selection UI (Select All/None), and Excel submission audit tracking
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1987,6 +1987,67 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TEST-APP-001</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Riot Games</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Gameplay Software Engineer</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>unity_gameplay.pdf</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Manual / Direct</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>https://riotgames.com/careers/123</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>https://riotgames.com/careers/123</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 17:23</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add interactive attached resume dropdown selectors across Discovered Jobs, JD Analyzer, and Excel Tracker
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -568,11 +568,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
+      <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -585,7 +581,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Phoenix Careers</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
@@ -597,7 +593,7 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 16:52</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr"/>
@@ -633,11 +629,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
+      <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -650,7 +642,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse (riotgames)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -666,7 +658,7 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:13</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr"/>
@@ -702,14 +694,10 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>68%</t>
-        </is>
-      </c>
+      <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>WAITING_FOR_USER</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -719,7 +707,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse (riotgames)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -735,7 +723,7 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:13</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr"/>
@@ -771,11 +759,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>89%</t>
-        </is>
-      </c>
+      <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -788,7 +772,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse (riotgames)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -804,7 +788,7 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:13</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr"/>
@@ -840,11 +824,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>76%</t>
-        </is>
-      </c>
+      <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -857,7 +837,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse (riotgames)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -873,7 +853,7 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:13</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr"/>
@@ -909,14 +889,10 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>45%</t>
-        </is>
-      </c>
+      <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -926,7 +902,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse (riotgames)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -942,7 +918,7 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:13</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr"/>
@@ -978,14 +954,10 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
+      <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>WAITING_FOR_USER</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -995,7 +967,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse (riotgames)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1011,7 +983,7 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:13</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr"/>
@@ -1047,14 +1019,10 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>74%</t>
-        </is>
-      </c>
+      <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>WAITING_FOR_USER</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1064,7 +1032,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse (riotgames)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1080,7 +1048,7 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:13</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr"/>
@@ -1116,11 +1084,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>89%</t>
-        </is>
-      </c>
+      <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1133,7 +1097,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse (riotgames)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1149,7 +1113,7 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:13</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr"/>
@@ -1185,11 +1149,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>76%</t>
-        </is>
-      </c>
+      <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1202,7 +1162,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse (riotgames)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1218,7 +1178,7 @@
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:13</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr"/>
@@ -1254,14 +1214,10 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>74%</t>
-        </is>
-      </c>
+      <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>WAITING_FOR_USER</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1271,7 +1227,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Greenhouse (riotgames)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1287,7 +1243,7 @@
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:13</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr"/>
@@ -1323,11 +1279,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>77%</t>
-        </is>
-      </c>
+      <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1340,7 +1292,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Web Page (https://remotegamejobs.com/)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1356,7 +1308,7 @@
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:14</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr"/>
@@ -1392,11 +1344,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>89%</t>
-        </is>
-      </c>
+      <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1409,7 +1357,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Web Page (https://remotegamejobs.com/)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1425,7 +1373,7 @@
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:14</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr"/>
@@ -1461,11 +1409,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>91%</t>
-        </is>
-      </c>
+      <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1478,7 +1422,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Web Page (https://remotegamejobs.com/)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1494,7 +1438,7 @@
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:14</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr"/>
@@ -1530,11 +1474,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>77%</t>
-        </is>
-      </c>
+      <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1547,7 +1487,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Web Page (https://remotegamejobs.com/)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1563,7 +1503,7 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:14</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
@@ -1599,11 +1539,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>91%</t>
-        </is>
-      </c>
+      <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1616,7 +1552,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Web Page (https://remotegamejobs.com/)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1632,7 +1568,7 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:14</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr"/>
@@ -1668,11 +1604,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>83%</t>
-        </is>
-      </c>
+      <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1685,7 +1617,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Web Page (https://remotegamejobs.com/)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1701,7 +1633,7 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:14</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
@@ -1737,11 +1669,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>77%</t>
-        </is>
-      </c>
+      <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1754,7 +1682,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Web Page (https://remotegamejobs.com/)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1770,7 +1698,7 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:14</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr"/>
@@ -1806,11 +1734,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>93%</t>
-        </is>
-      </c>
+      <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1823,7 +1747,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Web Page (https://remotegamejobs.com/)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1839,7 +1763,7 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:14</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr"/>
@@ -1875,11 +1799,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>91%</t>
-        </is>
-      </c>
+      <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1892,7 +1812,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Web Page (https://remotegamejobs.com/)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -1908,7 +1828,7 @@
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:14</t>
+          <t>2026-08-23 22:37</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
@@ -1944,11 +1864,7 @@
           <t>Full-time</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>98%</t>
-        </is>
-      </c>
+      <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1961,7 +1877,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Web Page (https://remotegamejobs.com/)</t>
+          <t>Manual / Direct</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1977,7 +1893,7 @@
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 17:14</t>
+          <t>2026-08-23 22:36</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr"/>
@@ -2042,11 +1958,68 @@
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:28</t>
+          <t>2026-08-23 22:43</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr"/>
       <c r="O23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>APP-LINK-COMM</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Community Guidelines</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Manual / Direct</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/help/linkedin/answer/34593?lang=en&amp;amp;trk=d_checkpoint_lg_consumer_login_ft_community_guidelines</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/help/linkedin/answer/34593?lang=en&amp;amp;trk=d_checkpoint_lg_consumer_login_ft_community_guidelines</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:36</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add responsive Stop and Cancel buttons with AbortControllers across Discovery, Applying, and Analysis
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -571,7 +571,7 @@
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -590,10 +590,14 @@
           <t>https://careers.phoenixinteractive.example.com/jobs/gameplay-programmer</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:49</t>
+        </is>
+      </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:49</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr"/>
@@ -632,7 +636,7 @@
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -655,10 +659,14 @@
           <t>https://www.riotgames.com/en/work-with-us/job/7977844?gh_jid=7977844</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:49</t>
+        </is>
+      </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:49</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr"/>
@@ -697,7 +705,7 @@
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -720,10 +728,14 @@
           <t>https://www.riotgames.com/en/work-with-us/job/8140324?gh_jid=8140324</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:49</t>
+        </is>
+      </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:49</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr"/>
@@ -762,7 +774,7 @@
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -785,10 +797,14 @@
           <t>https://www.riotgames.com/en/work-with-us/job/8112511?gh_jid=8112511</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:49</t>
+        </is>
+      </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:49</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr"/>
@@ -827,7 +843,7 @@
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -850,10 +866,14 @@
           <t>https://www.riotgames.com/en/work-with-us/job/8055923?gh_jid=8055923</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:49</t>
+        </is>
+      </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:49</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr"/>
@@ -892,7 +912,7 @@
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -915,10 +935,14 @@
           <t>https://www.riotgames.com/en/work-with-us/job/7424379?gh_jid=7424379</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:49</t>
+        </is>
+      </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:49</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr"/>
@@ -957,7 +981,7 @@
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -980,10 +1004,14 @@
           <t>https://www.riotgames.com/en/work-with-us/job/8118875?gh_jid=8118875</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:50</t>
+        </is>
+      </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:50</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr"/>
@@ -1022,7 +1050,7 @@
       <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1045,10 +1073,14 @@
           <t>https://www.riotgames.com/en/work-with-us/job/7905081?gh_jid=7905081</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:50</t>
+        </is>
+      </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:50</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr"/>
@@ -1087,7 +1119,7 @@
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1110,10 +1142,14 @@
           <t>https://www.riotgames.com/en/work-with-us/job/7982892?gh_jid=7982892</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:50</t>
+        </is>
+      </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:50</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr"/>
@@ -1152,7 +1188,7 @@
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1175,10 +1211,14 @@
           <t>https://www.riotgames.com/en/work-with-us/job/8129450?gh_jid=8129450</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:50</t>
+        </is>
+      </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:50</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr"/>
@@ -1217,7 +1257,7 @@
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1240,10 +1280,14 @@
           <t>https://www.riotgames.com/en/work-with-us/job/8082836?gh_jid=8082836</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:50</t>
+        </is>
+      </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:50</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr"/>
@@ -1282,7 +1326,7 @@
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1305,10 +1349,14 @@
           <t>https://remotegamejobs.com/remote-game-community-management-jobs</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:50</t>
+        </is>
+      </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:50</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr"/>
@@ -1347,7 +1395,7 @@
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1370,10 +1418,14 @@
           <t>https://remotegamejobs.com/jobs/telescope-games-senior-game-engineer-systems-engine-remote-job</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:50</t>
+        </is>
+      </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:50</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr"/>
@@ -1412,7 +1464,7 @@
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1435,10 +1487,14 @@
           <t>https://remotegamejobs.com/jobs/crytivo-qa-tester-remote-game-jobs-remote-job</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:50</t>
+        </is>
+      </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:50</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr"/>
@@ -1477,7 +1533,7 @@
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1500,10 +1556,14 @@
           <t>https://remotegamejobs.com/jobs/unfold-games-3d-character-animator-humanoid-animation-remote-job</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:50</t>
+        </is>
+      </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:50</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
@@ -1542,7 +1602,7 @@
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1565,10 +1625,14 @@
           <t>https://remotegamejobs.com/jobs/seismic-squirrel-senior-videogame-tester-remote-remote-job</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:50</t>
+        </is>
+      </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:50</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr"/>
@@ -1607,7 +1671,7 @@
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1630,10 +1694,14 @@
           <t>https://remotegamejobs.com/jobs/seismic-squirrel-senior-unity-technical-artist-remote-remote-job</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:50</t>
+        </is>
+      </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:50</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
@@ -1672,7 +1740,7 @@
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1695,10 +1763,14 @@
           <t>https://remotegamejobs.com/jobs/speedway-games-junior-vehicle-artist-remote-job-20abfac0-ec88-45bc-908e-f359a25648bb</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:51</t>
+        </is>
+      </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:51</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr"/>
@@ -1737,7 +1809,7 @@
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1760,10 +1832,14 @@
           <t>https://remotegamejobs.com/jobs/smile-break-senior-game-designer-combat-remote-job</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:51</t>
+        </is>
+      </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:51</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr"/>
@@ -1802,7 +1878,7 @@
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1825,10 +1901,14 @@
           <t>https://remotegamejobs.com/jobs/smile-break-senior-game-server-engineer-remote-job</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:51</t>
+        </is>
+      </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:37</t>
+          <t>2026-08-23 22:51</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
@@ -1867,7 +1947,7 @@
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1890,10 +1970,14 @@
           <t>https://remotegamejobs.com/jobs/mysteria-studio-ug-gameplay-programmer-intern-remote-job</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:51</t>
+        </is>
+      </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:51</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr"/>
@@ -1958,7 +2042,7 @@
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:43</t>
+          <t>2026-08-23 22:52</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr"/>
@@ -1993,7 +2077,7 @@
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>APPLIED</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -2012,10 +2096,14 @@
           <t>https://www.linkedin.com/help/linkedin/answer/34593?lang=en&amp;amp;trk=d_checkpoint_lg_consumer_login_ft_community_guidelines</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 22:51</t>
+        </is>
+      </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:36</t>
+          <t>2026-08-23 22:51</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Sync updated tracker.xlsx dataset
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -592,12 +592,12 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:49</t>
+          <t>2026-08-23 22:53</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 22:49</t>
+          <t>2026-08-23 22:53</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
fix: resolve MatchScoreBreakdown validation errors by adding default values and explicit kwargs in generate_drafts
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2042,7 +2042,7 @@
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 09:00</t>
+          <t>2026-08-24 09:23</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr"/>
@@ -2108,6 +2108,420 @@
       </c>
       <c r="N24" s="2" t="inlineStr"/>
       <c r="O24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>APP-920FA6CB</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Packsify</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Community &amp; Partner Lead</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>57%</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>SaiKowsikAyyalasomayajulaResume.pdf</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>RemoteGameJobs</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>https://remotegamejobs.com/jobs/packsify-llc-community-partner-manager-remote-job</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>https://remotegamejobs.com/jobs/packsify-llc-community-partner-manager-remote-job</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24 09:11</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>Overall Match: 57.0% | Status: REJECT. Role 'Community &amp; Partner Lead' at Packsify matches 1 key candidate areas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>APP-C5BBC728</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Tanglewood Games</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Technical Artist</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>76%</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>SaiKowsikAyyalasomayajulaResume.pdf</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>RemoteGameJobs</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>https://remotegamejobs.com/jobs/tanglewood-games-open-application-tech-art-remote-job</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>https://remotegamejobs.com/jobs/tanglewood-games-open-application-tech-art-remote-job</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24 09:11</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Overall Match: 76.0% | Status: AUTO_APPLY. Role 'Technical Artist' at Tanglewood Games matches 3 key candidate areas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>APP-3C444345</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Unknown Worlds</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Senior Technical Animator</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>77%</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>SaiKowsikAyyalasomayajulaResume.pdf</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>RemoteGameJobs</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>https://remotegamejobs.com/jobs/unknown-worlds-senior-technical-animator-remote-job</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>https://remotegamejobs.com/jobs/unknown-worlds-senior-technical-animator-remote-job</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24 09:12</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>Overall Match: 77.0% | Status: AUTO_APPLY. Role 'Senior Technical Animator' at Unknown Worlds matches 3 key candidate areas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>APP-D7B4E0BC</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Applied Intuition</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>77%</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>SaiKowsikAyyalasomayajulaResume.pdf</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Fetchrss</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/applied-intuition-inc?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/applied-intuition-inc?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24 09:12</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Overall Match: 77.0% | Status: AUTO_APPLY. Role 'Unknown' at Applied Intuition matches 1 key candidate areas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>APP-B2BB9C87</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Nex</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>77%</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>SaiKowsikAyyalasomayajulaResume.pdf</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Fetchrss</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/nexinc?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/nexinc?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24 09:12</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>Overall Match: 77.0% | Status: AUTO_APPLY. Role 'Unknown' at Nex matches 1 key candidate areas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>APP-2C234171</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>KOMODO Co., Ltd.</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>77%</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>SaiKowsikAyyalasomayajulaResume.pdf</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Fetchrss</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>https://jp.linkedin.com/company/komodo-co-ltd?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>https://jp.linkedin.com/company/komodo-co-ltd?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24 09:12</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>Overall Match: 77.0% | Status: AUTO_APPLY. Role 'Unknown' at KOMODO Co., Ltd. matches 1 key candidate areas.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>